<commit_message>
feat: Use Google Sheets API with secure environment variables
</commit_message>
<xml_diff>
--- a/teams.xlsx
+++ b/teams.xlsx
@@ -397,10 +397,99 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1"/>
-  <sheetData/>
+  <dimension ref="A1:T2"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>id</v>
+      </c>
+      <c r="B1" t="str">
+        <v>name</v>
+      </c>
+      <c r="C1" t="str">
+        <v>domain</v>
+      </c>
+      <c r="D1" t="str">
+        <v>members</v>
+      </c>
+      <c r="E1" t="str">
+        <v>isProblemStatementLocked</v>
+      </c>
+      <c r="F1" t="str">
+        <v>isRound1Locked</v>
+      </c>
+      <c r="G1" t="str">
+        <v>isRound2Locked</v>
+      </c>
+      <c r="H1" t="str">
+        <v>isRound3Locked</v>
+      </c>
+      <c r="I1" t="str">
+        <v>r1_1</v>
+      </c>
+      <c r="J1" t="str">
+        <v>r1_2</v>
+      </c>
+      <c r="K1" t="str">
+        <v>r1_3</v>
+      </c>
+      <c r="L1" t="str">
+        <v>r1_4</v>
+      </c>
+      <c r="M1" t="str">
+        <v>r2_1</v>
+      </c>
+      <c r="N1" t="str">
+        <v>r2_2</v>
+      </c>
+      <c r="O1" t="str">
+        <v>r2_3</v>
+      </c>
+      <c r="P1" t="str">
+        <v>r2_4</v>
+      </c>
+      <c r="Q1" t="str">
+        <v>r3_1</v>
+      </c>
+      <c r="R1" t="str">
+        <v>r3_2</v>
+      </c>
+      <c r="S1" t="str">
+        <v>r3_3</v>
+      </c>
+      <c r="T1" t="str">
+        <v>r3_4</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>T-1234</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Test Team</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Web</v>
+      </c>
+      <c r="D2" t="str">
+        <v/>
+      </c>
+      <c r="E2" t="b">
+        <v>0</v>
+      </c>
+      <c r="F2" t="b">
+        <v>0</v>
+      </c>
+      <c r="G2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:T2"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: migrate from Google Sheets to AWS RDS PostgreSQL
</commit_message>
<xml_diff>
--- a/teams.xlsx
+++ b/teams.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:T2"/>
+  <dimension ref="A1:T3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -487,9 +487,20 @@
         <v>0</v>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>RDS-001</v>
+      </c>
+      <c r="B3" t="str">
+        <v>RDS DB Test</v>
+      </c>
+      <c r="C3" t="str">
+        <v>AI</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:T2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:T3"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>